<commit_message>
build; correct missing ;
</commit_message>
<xml_diff>
--- a/classification-systems/nzlum/build/nzlum_v0.4.0.xlsx
+++ b/classification-systems/nzlum/build/nzlum_v0.4.0.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1383,50 +1383,50 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>2.9.0</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Smallholder farm</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>3.0.0</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Built environment</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>3.1.0</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Residential</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>3.1.1</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>High-density residential</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>3.1.2</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>Medium-density residential</t>
         </is>
       </c>
     </row>
@@ -1437,12 +1437,12 @@
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>3.1.3</t>
+          <t>3.1.2</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Low-density residential</t>
+          <t>Medium-density residential</t>
         </is>
       </c>
     </row>
@@ -1453,52 +1453,52 @@
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>3.1.3</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Rural residential</t>
+          <t>Low-density residential</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
       <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>3.2.0</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Public recreation and services</t>
-        </is>
-      </c>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>3.2.1</t>
+          <t>3.1.4</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Outdoor recreation</t>
+          <t>Rural residential</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
       <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="n"/>
-      <c r="D57" s="2" t="n"/>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>3.2.0</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Public recreation and services</t>
+        </is>
+      </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>3.2.2</t>
+          <t>3.2.1</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Indoor recreation</t>
+          <t>Outdoor recreation</t>
         </is>
       </c>
     </row>
@@ -1509,52 +1509,52 @@
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>3.2.3</t>
+          <t>3.2.2</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Community services</t>
+          <t>Indoor recreation</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
       <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>3.3.0</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>3.3.1</t>
+          <t>3.2.3</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Community services</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
       <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="n"/>
-      <c r="D60" s="2" t="n"/>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>3.3.0</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>3.3.2</t>
+          <t>3.3.1</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Retail</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>3.3.3</t>
+          <t>3.3.2</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Hospitality</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1581,12 @@
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>3.3.4</t>
+          <t>3.3.3</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Hospitality</t>
         </is>
       </c>
     </row>
@@ -1597,12 +1597,12 @@
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>3.3.5</t>
+          <t>3.3.4</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Entertainment</t>
         </is>
       </c>
     </row>
@@ -1613,52 +1613,52 @@
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>3.3.6</t>
+          <t>3.3.5</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Transportation &amp; warehousing</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
       <c r="B65" s="2" t="n"/>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>3.4.0</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>Manufacturing and industrial</t>
-        </is>
-      </c>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>3.4.1</t>
+          <t>3.3.6</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>General purpose factory</t>
+          <t>Transportation &amp; warehousing</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
       <c r="B66" s="2" t="n"/>
-      <c r="C66" s="2" t="n"/>
-      <c r="D66" s="2" t="n"/>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>3.4.0</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing and industrial</t>
+        </is>
+      </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>3.4.2</t>
+          <t>3.4.1</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Food processing factory</t>
+          <t>General purpose factory</t>
         </is>
       </c>
     </row>
@@ -1669,12 +1669,12 @@
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>3.4.3</t>
+          <t>3.4.2</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Major industrial complex</t>
+          <t>Food processing factory</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>3.4.4</t>
+          <t>3.4.3</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Sawmill</t>
+          <t>Major industrial complex</t>
         </is>
       </c>
     </row>
@@ -1701,12 +1701,12 @@
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>3.4.5</t>
+          <t>3.4.4</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Farm buildings/infrastructure</t>
+          <t>Sawmill</t>
         </is>
       </c>
     </row>
@@ -1717,52 +1717,52 @@
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>3.4.6</t>
+          <t>3.4.5</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Abattoirs</t>
+          <t>Farm buildings/infrastructure</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
       <c r="B71" s="2" t="n"/>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>3.5.0</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>Utilities</t>
-        </is>
-      </c>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>3.5.1</t>
+          <t>3.4.6</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Fuel powered electricity generation</t>
+          <t>Abattoirs</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
       <c r="B72" s="2" t="n"/>
-      <c r="C72" s="2" t="n"/>
-      <c r="D72" s="2" t="n"/>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>3.5.0</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>3.5.2</t>
+          <t>3.5.1</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Hydroelectricity generation</t>
+          <t>Fuel powered electricity generation</t>
         </is>
       </c>
     </row>
@@ -1773,12 +1773,12 @@
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>3.5.3</t>
+          <t>3.5.2</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Wind electricity generation</t>
+          <t>Hydroelectricity generation</t>
         </is>
       </c>
     </row>
@@ -1789,12 +1789,12 @@
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>3.5.4</t>
+          <t>3.5.3</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Solar electricity generation</t>
+          <t>Wind electricity generation</t>
         </is>
       </c>
     </row>
@@ -1805,12 +1805,12 @@
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>3.5.5</t>
+          <t>3.5.4</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Electricity substations and transmission</t>
+          <t>Solar electricity generation</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>3.5.6</t>
+          <t>3.5.5</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Gas treatment, storage, and transmission</t>
+          <t>Electricity substations and transmission</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1837,12 @@
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>3.5.7</t>
+          <t>3.5.6</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Water extraction and transmission</t>
+          <t>Gas treatment, storage, and transmission</t>
         </is>
       </c>
     </row>
@@ -1853,52 +1853,52 @@
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>3.5.8</t>
+          <t>3.5.7</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Navigation and communication</t>
+          <t>Water extraction and transmission</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
       <c r="B79" s="2" t="n"/>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>3.6.0</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>3.6.1</t>
+          <t>3.5.8</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Airports/aerodromes</t>
+          <t>Navigation and communication</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
       <c r="B80" s="2" t="n"/>
-      <c r="C80" s="2" t="n"/>
-      <c r="D80" s="2" t="n"/>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>3.6.0</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>3.6.2</t>
+          <t>3.6.1</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Roads</t>
+          <t>Airports/aerodromes</t>
         </is>
       </c>
     </row>
@@ -1909,12 +1909,12 @@
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>3.6.3</t>
+          <t>3.6.2</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Railways</t>
+          <t>Roads</t>
         </is>
       </c>
     </row>
@@ -1925,52 +1925,52 @@
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>3.6.4</t>
+          <t>3.6.3</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Ports and water transport</t>
+          <t>Railways</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
       <c r="B83" s="2" t="n"/>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>3.7.0</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>Mining</t>
-        </is>
-      </c>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>3.7.1</t>
+          <t>3.6.4</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Mines</t>
+          <t>Ports and water transport</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
       <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="n"/>
-      <c r="D84" s="2" t="n"/>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>3.7.0</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Mining</t>
+        </is>
+      </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>3.7.2</t>
+          <t>3.7.1</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Quarries</t>
+          <t>Mines</t>
         </is>
       </c>
     </row>
@@ -1981,12 +1981,12 @@
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>3.7.3</t>
+          <t>3.7.2</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Tailings</t>
+          <t>Quarries</t>
         </is>
       </c>
     </row>
@@ -1997,12 +1997,12 @@
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>3.7.4</t>
+          <t>3.7.3</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Evaporation basins</t>
+          <t>Tailings</t>
         </is>
       </c>
     </row>
@@ -2013,52 +2013,52 @@
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>3.7.5</t>
+          <t>3.7.4</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Extractive industry not in use</t>
+          <t>Evaporation basins</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
       <c r="B88" s="2" t="n"/>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>3.8.0</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>Waste treatment and disposal</t>
-        </is>
-      </c>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>3.8.1</t>
+          <t>3.7.5</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Landfills</t>
+          <t>Extractive industry not in use</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
       <c r="B89" s="2" t="n"/>
-      <c r="C89" s="2" t="n"/>
-      <c r="D89" s="2" t="n"/>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>3.8.0</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Waste treatment and disposal</t>
+        </is>
+      </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>3.8.2</t>
+          <t>3.8.1</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Transfer stations and recycling facilities</t>
+          <t>Landfills</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>3.8.3</t>
+          <t>3.8.2</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Municipal wastewater</t>
+          <t>Transfer stations and recycling facilities</t>
         </is>
       </c>
     </row>
@@ -2085,12 +2085,12 @@
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>3.8.4</t>
+          <t>3.8.3</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Wastewater treatment – land application</t>
+          <t>Municipal wastewater</t>
         </is>
       </c>
     </row>
@@ -2101,52 +2101,52 @@
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>3.8.5</t>
+          <t>3.8.4</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Stormwater management</t>
+          <t>Wastewater treatment – land application</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
       <c r="B93" s="2" t="n"/>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>3.9.0</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>Vacant and transitioning land</t>
-        </is>
-      </c>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>3.9.1</t>
+          <t>3.8.5</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Brownfield development</t>
+          <t>Stormwater management</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
       <c r="B94" s="2" t="n"/>
-      <c r="C94" s="2" t="n"/>
-      <c r="D94" s="2" t="n"/>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>3.9.0</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Vacant and transitioning land</t>
+        </is>
+      </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>3.9.2</t>
+          <t>3.9.1</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Greenfield development</t>
+          <t>Brownfield development</t>
         </is>
       </c>
     </row>
@@ -2157,10 +2157,26 @@
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="inlineStr">
         <is>
+          <t>3.9.2</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Greenfield development</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="2" t="n"/>
+      <c r="C96" s="2" t="n"/>
+      <c r="D96" s="2" t="n"/>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
           <t>3.9.3</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
+      <c r="F96" s="2" t="inlineStr">
         <is>
           <t>Idle and derelict land</t>
         </is>
@@ -2168,52 +2184,52 @@
     </row>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="C56:C58"/>
-    <mergeCell ref="D56:D58"/>
     <mergeCell ref="D22:D25"/>
-    <mergeCell ref="B52:B95"/>
+    <mergeCell ref="C57:C59"/>
+    <mergeCell ref="D60:D65"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="C43:C47"/>
     <mergeCell ref="C29:C32"/>
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="C2:C8"/>
-    <mergeCell ref="D93:D95"/>
+    <mergeCell ref="D80:D83"/>
     <mergeCell ref="D36:D37"/>
-    <mergeCell ref="D59:D64"/>
-    <mergeCell ref="C79:C82"/>
-    <mergeCell ref="B22:B51"/>
     <mergeCell ref="D9:D11"/>
     <mergeCell ref="D43:D47"/>
-    <mergeCell ref="D65:D70"/>
     <mergeCell ref="C22:C25"/>
-    <mergeCell ref="D52:D55"/>
-    <mergeCell ref="D83:D87"/>
     <mergeCell ref="A2:A21"/>
     <mergeCell ref="D26:D28"/>
     <mergeCell ref="D48:D51"/>
     <mergeCell ref="C38:C42"/>
-    <mergeCell ref="C65:C70"/>
     <mergeCell ref="D38:D42"/>
+    <mergeCell ref="D89:D93"/>
     <mergeCell ref="C33:C35"/>
+    <mergeCell ref="D94:D96"/>
     <mergeCell ref="C36:C37"/>
-    <mergeCell ref="C59:C64"/>
-    <mergeCell ref="D88:D92"/>
-    <mergeCell ref="C52:C55"/>
+    <mergeCell ref="B53:B96"/>
+    <mergeCell ref="C80:C83"/>
+    <mergeCell ref="A22:A52"/>
+    <mergeCell ref="D84:D88"/>
+    <mergeCell ref="D66:D71"/>
+    <mergeCell ref="A53:A96"/>
     <mergeCell ref="C12:C19"/>
-    <mergeCell ref="C71:C78"/>
+    <mergeCell ref="D72:D79"/>
+    <mergeCell ref="C89:C93"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="D53:D56"/>
     <mergeCell ref="D20:D21"/>
-    <mergeCell ref="C83:C87"/>
-    <mergeCell ref="C93:C95"/>
     <mergeCell ref="C26:C28"/>
+    <mergeCell ref="B22:B52"/>
     <mergeCell ref="C48:C51"/>
-    <mergeCell ref="C88:C92"/>
-    <mergeCell ref="A52:A95"/>
-    <mergeCell ref="A22:A51"/>
+    <mergeCell ref="C72:C79"/>
+    <mergeCell ref="C60:C65"/>
+    <mergeCell ref="C66:C71"/>
     <mergeCell ref="D12:D19"/>
-    <mergeCell ref="D79:D82"/>
+    <mergeCell ref="D57:D59"/>
     <mergeCell ref="D29:D32"/>
-    <mergeCell ref="D71:D78"/>
+    <mergeCell ref="C84:C88"/>
     <mergeCell ref="D2:D8"/>
+    <mergeCell ref="C53:C56"/>
     <mergeCell ref="B2:B21"/>
     <mergeCell ref="C9:C11"/>
   </mergeCells>

</xml_diff>